<commit_message>
fix: update baseline password minimum length requirement from 14 to 21 characters
</commit_message>
<xml_diff>
--- a/Configuration_Baseline_Checklist.xlsx
+++ b/Configuration_Baseline_Checklist.xlsx
@@ -690,7 +690,7 @@
       </c>
       <c r="D5" s="9" t="inlineStr">
         <is>
-          <t>minlen=14, dcredit=-1, ucredit=-1, lcredit=-1, ocredit=-1, SHA512 algoritması. Root parolası asla e-posta/sohbet üzerinden paylaşılmamalıdır.</t>
+          <t>minlen=21, dcredit=-1, ucredit=-1, lcredit=-1, ocredit=-1, SHA512 algoritması. Root parolası asla e-posta/sohbet üzerinden paylaşılmamalıdır.</t>
         </is>
       </c>
       <c r="E5" s="9" t="inlineStr">
@@ -1824,7 +1824,7 @@
       </c>
       <c r="D4" s="9" t="inlineStr">
         <is>
-          <t>En az 14 karakter, büyük/küçük harf, rakam ve özel karakter içermeli. Varsayılan "Administrator" hesabı yeniden adlandırılmalıdır.</t>
+          <t>En az 21 karakter, büyük/küçük harf, rakam ve özel karakter içermeli. Varsayılan "Administrator" hesabı yeniden adlandırılmalıdır.</t>
         </is>
       </c>
       <c r="E4" s="9" t="inlineStr">
@@ -2111,7 +2111,7 @@
       </c>
       <c r="D12" s="9" t="inlineStr">
         <is>
-          <t>Minimum uzunluk: 14 karakter. Karmaşıklık: Etkin. Maksimum yaş: 90 gün. Geçmiş: 24 şifre. Hesap kilitleme: 5 deneme / 15 dk.</t>
+          <t>Minimum uzunluk: 21 karakter. Karmaşıklık: Etkin. Maksimum yaş: 90 gün. Geçmiş: 24 şifre. Hesap kilitleme: 5 deneme / 15 dk.</t>
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr">
@@ -3865,7 +3865,7 @@
       </c>
       <c r="D13" s="9" t="inlineStr">
         <is>
-          <t>Karmaşıklık: Etkin. Minimum uzunluk: 14 karakter. Maksimum yaş: 90 gün. Geçmiş: 24 şifre. Kilitleme: 5 deneme / 15 dk.</t>
+          <t>Karmaşıklık: Etkin. Minimum uzunluk: 21 karakter. Maksimum yaş: 90 gün. Geçmiş: 24 şifre. Kilitleme: 5 deneme / 15 dk.</t>
         </is>
       </c>
       <c r="E13" s="9" t="inlineStr">

</xml_diff>